<commit_message>
Added MF to probes / probe sets
</commit_message>
<xml_diff>
--- a/phase2/june2026/RQ2-buckets.xlsx
+++ b/phase2/june2026/RQ2-buckets.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\darren.gemoets_cn\Documents\ITM\git\itm-ingest\phase2\june2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF7E9701-08E4-4653-8450-9342A8FE3B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3F8E407-9968-4840-9D88-D42089F80A7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{EE43EC17-22E9-4752-A5B2-870C3FD56D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{EE43EC17-22E9-4752-A5B2-870C3FD56D40}"/>
   </bookViews>
   <sheets>
     <sheet name="AF" sheetId="1" r:id="rId1"/>
-    <sheet name="PS" sheetId="3" r:id="rId2"/>
-    <sheet name="SS" sheetId="4" r:id="rId3"/>
+    <sheet name="MF" sheetId="5" r:id="rId2"/>
+    <sheet name="PS" sheetId="3" r:id="rId3"/>
+    <sheet name="SS" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="11">
   <si>
     <t>0.0370043, 0.054312911</t>
   </si>
@@ -65,6 +66,12 @@
   </si>
   <si>
     <t>Medical buckets</t>
+  </si>
+  <si>
+    <t>0.35372487, 0.39072917, 0.392521776</t>
+  </si>
+  <si>
+    <t>0.574049028, 0.575841634</t>
   </si>
 </sst>
 </file>
@@ -593,6 +600,158 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{090975FD-FA39-40FB-A973-3C0FAE629A04}">
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.5703125" style="1" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1">
+        <v>0.53704472800000003</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1">
+        <v>0.63015454500000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>1</v>
+      </c>
+      <c r="B11" s="1">
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>2</v>
+      </c>
+      <c r="B12" s="1">
+        <v>0.17100000000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>3</v>
+      </c>
+      <c r="B13" s="1">
+        <v>0.32950000000000002</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>5</v>
+      </c>
+      <c r="B15" s="1">
+        <v>0.48049999999999998</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>6</v>
+      </c>
+      <c r="B16" s="1">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>7</v>
+      </c>
+      <c r="B17" s="1">
+        <v>0.84450000000000003</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01C585B0-5742-4A0B-B930-C8653EBD7191}">
   <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -732,7 +891,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40482F60-53AF-44C4-972A-1C9A9AD5BF50}">
   <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>